<commit_message>
M1-302: add review request and update backlog status
- GPT_REVIEW_REQUEST_M1-302.md for the cross-model review round.
- M1-302 -> In Review in backlog.csv and the .xlsx.
- M1-301 -> Done: it merged as PR #6, and per the status vocabulary an item
  becomes Done at merge, not when the code lands.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/whiskeyjack-bot-v1-backlog.xlsx
+++ b/whiskeyjack-bot-v1-backlog.xlsx
@@ -788,7 +788,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="43" t="inlineStr">
         <is>
@@ -1635,7 +1634,7 @@
       </c>
       <c r="J18" s="31" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K18" s="32" t="inlineStr">
@@ -1692,7 +1691,7 @@
       </c>
       <c r="J19" s="31" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="K19" s="32" t="inlineStr">

</xml_diff>

<commit_message>
docs: mark M1-202 Done, and M1-203 In Review
Two separate corrections to the backlog, in both the CSV and the xlsx.

M1-202 was left at `In Review` when PR #8 merged. The status vocabulary is
explicit that `Done` happens at merge, not when the code lands, so master has
been misreporting a merged item since 3620d46.

M1-203 moves to `In Review` as its PR opens.

Both xlsx edits patch the single inline-string cell (Backlog!J16, Backlog!J17)
inside the zip rather than round-tripping through openpyxl, so the other 19
parts stay byte-identical: the workbook carries conditional formatting, merged
cells and named tables that a rewrite can silently damage.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/whiskeyjack-bot-v1-backlog.xlsx
+++ b/whiskeyjack-bot-v1-backlog.xlsx
@@ -1521,7 +1521,7 @@
       </c>
       <c r="J16" s="31" t="inlineStr">
         <is>
-          <t>In Review</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K16" s="32" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="J17" s="31" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="K17" s="32" t="inlineStr">

</xml_diff>

<commit_message>
chore: sync backlog xlsx with CSV status column
The xlsx mirror had drifted from docs/backlog/backlog.csv — several Done-at-merge
flips were only ever applied to the CSV. Bring the six stale status cells into
line so the two sources agree (CLAUDE.md requires updating both):

- M1-201 In Review -> Done   (merged #4; xlsx flip was missed)
- M1-203 In Review -> Done   (merged #10)
- M1-301 Not Started -> Done       (merged #6)
- M1-401 Not Started -> Done       (merged #9/#11)
- M1-302 Not Started -> In Review   (approved #7, awaiting merge)
- M1-305 Not Started -> In Review   (in development #12)

Only xl/worksheets/sheet1.xml (inline-string status cells in column J) changed;
all other archive members are byte-identical. No CSV change — the CSV is already
correct as of #10.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/whiskeyjack-bot-v1-backlog.xlsx
+++ b/whiskeyjack-bot-v1-backlog.xlsx
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J15" s="31" t="inlineStr">
         <is>
-          <t>In Review</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K15" s="32" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="J17" s="31" t="inlineStr">
         <is>
-          <t>In Review</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K17" s="32" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="J18" s="31" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K18" s="32" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="J19" s="31" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="K19" s="32" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="J22" s="31" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="K22" s="32" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="J24" s="31" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K24" s="32" t="inlineStr">

</xml_diff>